<commit_message>
Elmorry Ex4A insert records
</commit_message>
<xml_diff>
--- a/Elmorry_Ex3A_tables.xlsx
+++ b/Elmorry_Ex3A_tables.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30613"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{815A3CFE-7EA9-403F-AC23-1478A927B211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{395E5546-0684-4C1C-A73C-5A1E8DDFA3AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Customers" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
   <si>
     <t>customer_id</t>
   </si>
@@ -54,6 +54,18 @@
     <t>address</t>
   </si>
   <si>
+    <t>Maria Lopez</t>
+  </si>
+  <si>
+    <t>201-555-0142</t>
+  </si>
+  <si>
+    <t>maria.lopez@email.com</t>
+  </si>
+  <si>
+    <t>45 Oak Street, Secaucus, NJ</t>
+  </si>
+  <si>
     <t>dog_id</t>
   </si>
   <si>
@@ -72,6 +84,18 @@
     <t>emergency_contact_phone</t>
   </si>
   <si>
+    <t>Buddy</t>
+  </si>
+  <si>
+    <t>Golden Retriever</t>
+  </si>
+  <si>
+    <t>Carlos Lopez</t>
+  </si>
+  <si>
+    <t>201-555-0199</t>
+  </si>
+  <si>
     <t>appointment_id</t>
   </si>
   <si>
@@ -100,16 +124,30 @@
   </si>
   <si>
     <t>payment_status</t>
+  </si>
+  <si>
+    <t>Venmo</t>
+  </si>
+  <si>
+    <t>Paid</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -167,22 +205,27 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -495,14 +538,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.28515625" customWidth="1"/>
+    <col min="5" max="5" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1">
@@ -522,19 +565,39 @@
         <v>4</v>
       </c>
     </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{57CB713F-91C6-4C6E-A3B0-8A8FC9E9515A}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF16B271-0699-4CDC-AA4B-E9F0AD67F650}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="4.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
@@ -543,25 +606,48 @@
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +657,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E23771AD-B537-4653-B273-BAE2D003A03B}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
@@ -584,22 +670,42 @@
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>15</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="5">
+        <v>46321</v>
+      </c>
+      <c r="D2" s="6">
+        <v>0.375</v>
+      </c>
+      <c r="E2">
+        <v>30</v>
+      </c>
+      <c r="F2">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -609,7 +715,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8075DD8-4D3F-4DE9-81B9-CD7E99882CD1}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
@@ -622,22 +728,42 @@
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>25</v>
+      </c>
+      <c r="D2" s="5">
+        <v>46321</v>
+      </c>
+      <c r="E2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>